<commit_message>
feat: show completion percentage next to project names in missing reports panel
- Read column F (completion %) from 'new map data source04' sheet
- Display percentage in parentheses next to each project name
- Add styling for completion percentage in both dark and aegov themes
</commit_message>
<xml_diff>
--- a/chair man map assets/suggestion 01.xlsx
+++ b/chair man map assets/suggestion 01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ahmed Elsherbiny\AI PROJECTS\APPs PROJECTS\FOLLOW-UP APPLICATION OVERSEAS ONLINE DASHBOARD\chair man map assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BE825E-5255-4B63-BE43-F115FA6E1FA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14ED219B-868F-4D4A-83F5-2688C1676342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1099,12 +1099,11 @@
   <cols>
     <col min="1" max="1" width="3.8984375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="46.8984375" style="1"/>
-    <col min="3" max="3" width="9.09765625" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="21.5" style="1" hidden="1" customWidth="1"/>
-    <col min="6" max="7" width="43.09765625" style="1" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="46.09765625" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="9.09765625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="21.5" style="1" customWidth="1"/>
+    <col min="6" max="7" width="43.09765625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="46.8984375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="46.09765625" style="1" customWidth="1"/>
     <col min="10" max="16384" width="46.8984375" style="1"/>
   </cols>
   <sheetData>

</xml_diff>